<commit_message>
feat: remove loops from ast manual direct
</commit_message>
<xml_diff>
--- a/Horario_TV_Directo.xlsx
+++ b/Horario_TV_Directo.xlsx
@@ -2821,7 +2821,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>SERIE JUVENIL “SABRINA, LA BRUJA ADOLESCENTE”</t>
+          <t>SERIE JUVENIL “SABRINA…”</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -3484,11 +3484,7 @@
           <t>16:00</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
+      <c r="E2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3507,11 +3503,7 @@
           <t>19:30</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
+      <c r="E3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3530,11 +3522,7 @@
           <t>19:45</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>23:47</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3553,11 +3541,7 @@
           <t>16:00</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
+      <c r="E5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3576,11 +3560,7 @@
           <t>16:30</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3599,11 +3579,7 @@
           <t>16:00</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
+      <c r="E7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3622,11 +3598,7 @@
           <t>02:00</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>23:55</t>
-        </is>
-      </c>
+      <c r="E8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: update ast nodes
</commit_message>
<xml_diff>
--- a/Horario_TV_Directo.xlsx
+++ b/Horario_TV_Directo.xlsx
@@ -37,7 +37,7 @@
       <color rgb="00000000"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -50,42 +50,6 @@
         <bgColor rgb="FF4A90E2"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE6B8AF"/>
-        <bgColor rgb="FFE6B8AF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
-        <bgColor rgb="FFD9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA9D18E"/>
-        <bgColor rgb="FFA9D18E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB4C7E7"/>
-        <bgColor rgb="FFB4C7E7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFA500"/>
-        <bgColor rgb="FFFFA500"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFD966"/>
-        <bgColor rgb="FFFFD966"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -96,35 +60,29 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB7B7B7"/>
+      <left style="thick">
+        <color rgb="FF4F81BD"/>
       </left>
-      <right style="thin">
-        <color rgb="FFB7B7B7"/>
+      <right style="thick">
+        <color rgb="FF4F81BD"/>
       </right>
-      <top style="thin">
-        <color rgb="FFB7B7B7"/>
+      <top style="thick">
+        <color rgb="FF4F81BD"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FFB7B7B7"/>
+      <bottom style="thick">
+        <color rgb="FF4F81BD"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,7 +457,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -533,16 +491,16 @@
           <t>Tipo Calc</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
@@ -562,19 +520,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <f>IF(A3&lt;&gt;"",IF(ROW()=3,$G2,E2),"")</f>
         <v/>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <f>IF(A3&lt;&gt;"",TEXT(TIMEVALUE(D3)+(IFERROR(VLOOKUP(A3,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="2">
         <f>IF(A3&lt;&gt;"",IFERROR(VLOOKUP(A3,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -590,19 +547,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <f>IF(A4&lt;&gt;"",IF(ROW()=3,$G2,E3),"")</f>
         <v/>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <f>IF(A4&lt;&gt;"",TEXT(TIMEVALUE(D4)+(IFERROR(VLOOKUP(A4,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="2">
         <f>IF(A4&lt;&gt;"",IFERROR(VLOOKUP(A4,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -618,19 +574,18 @@
           <t>revista</t>
         </is>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="2">
         <f>IF(A5&lt;&gt;"",IF(ROW()=3,$G2,E4),"")</f>
         <v/>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="2">
         <f>IF(A5&lt;&gt;"",TEXT(TIMEVALUE(D5)+(IFERROR(VLOOKUP(A5,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="2">
         <f>IF(A5&lt;&gt;"",IFERROR(VLOOKUP(A5,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -646,19 +601,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="2">
         <f>IF(A6&lt;&gt;"",IF(ROW()=3,$G2,E5),"")</f>
         <v/>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="2">
         <f>IF(A6&lt;&gt;"",TEXT(TIMEVALUE(D6)+(IFERROR(VLOOKUP(A6,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="2">
         <f>IF(A6&lt;&gt;"",IFERROR(VLOOKUP(A6,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -674,19 +628,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="2">
         <f>IF(A7&lt;&gt;"",IF(ROW()=3,$G2,E6),"")</f>
         <v/>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="2">
         <f>IF(A7&lt;&gt;"",TEXT(TIMEVALUE(D7)+(IFERROR(VLOOKUP(A7,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="2">
         <f>IF(A7&lt;&gt;"",IFERROR(VLOOKUP(A7,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -702,19 +655,18 @@
           <t>infantil</t>
         </is>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="2">
         <f>IF(A8&lt;&gt;"",IF(ROW()=3,$G2,E7),"")</f>
         <v/>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="2">
         <f>IF(A8&lt;&gt;"",TEXT(TIMEVALUE(D8)+(IFERROR(VLOOKUP(A8,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="2">
         <f>IF(A8&lt;&gt;"",IFERROR(VLOOKUP(A8,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -730,19 +682,18 @@
           <t>cine</t>
         </is>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="2">
         <f>IF(A9&lt;&gt;"",IF(ROW()=3,$G2,E8),"")</f>
         <v/>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="2">
         <f>IF(A9&lt;&gt;"",TEXT(TIMEVALUE(D9)+(IFERROR(VLOOKUP(A9,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="2">
         <f>IF(A9&lt;&gt;"",IFERROR(VLOOKUP(A9,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -758,19 +709,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="2">
         <f>IF(A10&lt;&gt;"",IF(ROW()=3,$G2,E9),"")</f>
         <v/>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="2">
         <f>IF(A10&lt;&gt;"",TEXT(TIMEVALUE(D10)+(IFERROR(VLOOKUP(A10,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="2">
         <f>IF(A10&lt;&gt;"",IFERROR(VLOOKUP(A10,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -786,19 +736,18 @@
           <t>cine</t>
         </is>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="2">
         <f>IF(A11&lt;&gt;"",IF(ROW()=3,$G2,E10),"")</f>
         <v/>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="2">
         <f>IF(A11&lt;&gt;"",TEXT(TIMEVALUE(D11)+(IFERROR(VLOOKUP(A11,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="2">
         <f>IF(A11&lt;&gt;"",IFERROR(VLOOKUP(A11,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -814,19 +763,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="2">
         <f>IF(A12&lt;&gt;"",IF(ROW()=3,$G2,E11),"")</f>
         <v/>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="2">
         <f>IF(A12&lt;&gt;"",TEXT(TIMEVALUE(D12)+(IFERROR(VLOOKUP(A12,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="2">
         <f>IF(A12&lt;&gt;"",IFERROR(VLOOKUP(A12,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -842,19 +790,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="2">
         <f>IF(A13&lt;&gt;"",IF(ROW()=3,$G2,E12),"")</f>
         <v/>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="2">
         <f>IF(A13&lt;&gt;"",TEXT(TIMEVALUE(D13)+(IFERROR(VLOOKUP(A13,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="2">
         <f>IF(A13&lt;&gt;"",IFERROR(VLOOKUP(A13,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -870,19 +817,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="2">
         <f>IF(A14&lt;&gt;"",IF(ROW()=3,$G2,E13),"")</f>
         <v/>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="2">
         <f>IF(A14&lt;&gt;"",TEXT(TIMEVALUE(D14)+(IFERROR(VLOOKUP(A14,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="2">
         <f>IF(A14&lt;&gt;"",IFERROR(VLOOKUP(A14,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -898,19 +844,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="2">
         <f>IF(A15&lt;&gt;"",IF(ROW()=3,$G2,E14),"")</f>
         <v/>
       </c>
-      <c r="E15" s="7">
+      <c r="E15" s="2">
         <f>IF(A15&lt;&gt;"",TEXT(TIMEVALUE(D15)+(IFERROR(VLOOKUP(A15,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="2">
         <f>IF(A15&lt;&gt;"",IFERROR(VLOOKUP(A15,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -926,19 +871,18 @@
           <t>entrevista</t>
         </is>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="2">
         <f>IF(A16&lt;&gt;"",IF(ROW()=3,$G2,E15),"")</f>
         <v/>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="2">
         <f>IF(A16&lt;&gt;"",TEXT(TIMEVALUE(D16)+(IFERROR(VLOOKUP(A16,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="2">
         <f>IF(A16&lt;&gt;"",IFERROR(VLOOKUP(A16,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -954,19 +898,18 @@
           <t>ficción</t>
         </is>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="2">
         <f>IF(A17&lt;&gt;"",IF(ROW()=3,$G2,E16),"")</f>
         <v/>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="2">
         <f>IF(A17&lt;&gt;"",TEXT(TIMEVALUE(D17)+(IFERROR(VLOOKUP(A17,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="2">
         <f>IF(A17&lt;&gt;"",IFERROR(VLOOKUP(A17,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -982,19 +925,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="2">
         <f>IF(A18&lt;&gt;"",IF(ROW()=3,$G2,E17),"")</f>
         <v/>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="2">
         <f>IF(A18&lt;&gt;"",TEXT(TIMEVALUE(D18)+(IFERROR(VLOOKUP(A18,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="2">
         <f>IF(A18&lt;&gt;"",IFERROR(VLOOKUP(A18,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1010,19 +952,18 @@
           <t>ficción</t>
         </is>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="2">
         <f>IF(A19&lt;&gt;"",IF(ROW()=3,$G2,E18),"")</f>
         <v/>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="2">
         <f>IF(A19&lt;&gt;"",TEXT(TIMEVALUE(D19)+(IFERROR(VLOOKUP(A19,$A3:$C19,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="2">
         <f>IF(A19&lt;&gt;"",IFERROR(VLOOKUP(A19,$A3:$C19,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G19" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1044,7 +985,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1078,16 +1019,16 @@
           <t>Tipo Calc</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
@@ -1107,19 +1048,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="2">
         <f>IF(A3&lt;&gt;"",IF(ROW()=3,$G2,E2),"")</f>
         <v/>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="2">
         <f>IF(A3&lt;&gt;"",TEXT(TIMEVALUE(D3)+(IFERROR(VLOOKUP(A3,$A3:$C11,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="2">
         <f>IF(A3&lt;&gt;"",IFERROR(VLOOKUP(A3,$A3:$C11,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1135,19 +1075,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="2">
         <f>IF(A4&lt;&gt;"",IF(ROW()=3,$G2,E3),"")</f>
         <v/>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="2">
         <f>IF(A4&lt;&gt;"",TEXT(TIMEVALUE(D4)+(IFERROR(VLOOKUP(A4,$A3:$C11,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="2">
         <f>IF(A4&lt;&gt;"",IFERROR(VLOOKUP(A4,$A3:$C11,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1163,19 +1102,18 @@
           <t>salud</t>
         </is>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="2">
         <f>IF(A5&lt;&gt;"",IF(ROW()=3,$G2,E4),"")</f>
         <v/>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="2">
         <f>IF(A5&lt;&gt;"",TEXT(TIMEVALUE(D5)+(IFERROR(VLOOKUP(A5,$A3:$C11,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="2">
         <f>IF(A5&lt;&gt;"",IFERROR(VLOOKUP(A5,$A3:$C11,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1191,19 +1129,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="2">
         <f>IF(A6&lt;&gt;"",IF(ROW()=3,$G2,E5),"")</f>
         <v/>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="2">
         <f>IF(A6&lt;&gt;"",TEXT(TIMEVALUE(D6)+(IFERROR(VLOOKUP(A6,$A3:$C11,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="2">
         <f>IF(A6&lt;&gt;"",IFERROR(VLOOKUP(A6,$A3:$C11,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1219,19 +1156,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="2">
         <f>IF(A7&lt;&gt;"",IF(ROW()=3,$G2,E6),"")</f>
         <v/>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="2">
         <f>IF(A7&lt;&gt;"",TEXT(TIMEVALUE(D7)+(IFERROR(VLOOKUP(A7,$A3:$C11,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="2">
         <f>IF(A7&lt;&gt;"",IFERROR(VLOOKUP(A7,$A3:$C11,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1247,19 +1183,18 @@
           <t>entrevista</t>
         </is>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="2">
         <f>IF(A8&lt;&gt;"",IF(ROW()=3,$G2,E7),"")</f>
         <v/>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="2">
         <f>IF(A8&lt;&gt;"",TEXT(TIMEVALUE(D8)+(IFERROR(VLOOKUP(A8,$A3:$C11,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="2">
         <f>IF(A8&lt;&gt;"",IFERROR(VLOOKUP(A8,$A3:$C11,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1275,19 +1210,18 @@
           <t>ficción</t>
         </is>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="2">
         <f>IF(A9&lt;&gt;"",IF(ROW()=3,$G2,E8),"")</f>
         <v/>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="2">
         <f>IF(A9&lt;&gt;"",TEXT(TIMEVALUE(D9)+(IFERROR(VLOOKUP(A9,$A3:$C11,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="2">
         <f>IF(A9&lt;&gt;"",IFERROR(VLOOKUP(A9,$A3:$C11,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1303,19 +1237,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="2">
         <f>IF(A10&lt;&gt;"",IF(ROW()=3,$G2,E9),"")</f>
         <v/>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="2">
         <f>IF(A10&lt;&gt;"",TEXT(TIMEVALUE(D10)+(IFERROR(VLOOKUP(A10,$A3:$C11,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="2">
         <f>IF(A10&lt;&gt;"",IFERROR(VLOOKUP(A10,$A3:$C11,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1331,19 +1264,18 @@
           <t>ficción</t>
         </is>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="2">
         <f>IF(A11&lt;&gt;"",IF(ROW()=3,$G2,E10),"")</f>
         <v/>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="2">
         <f>IF(A11&lt;&gt;"",TEXT(TIMEVALUE(D11)+(IFERROR(VLOOKUP(A11,$A3:$C11,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="2">
         <f>IF(A11&lt;&gt;"",IFERROR(VLOOKUP(A11,$A3:$C11,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G11" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1365,7 +1297,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1399,16 +1331,16 @@
           <t>Tipo Calc</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
@@ -1428,19 +1360,18 @@
           <t>cine</t>
         </is>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="2">
         <f>IF(A3&lt;&gt;"",IF(ROW()=3,$G2,E2),"")</f>
         <v/>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="2">
         <f>IF(A3&lt;&gt;"",TEXT(TIMEVALUE(D3)+(IFERROR(VLOOKUP(A3,$A3:$C9,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="2">
         <f>IF(A3&lt;&gt;"",IFERROR(VLOOKUP(A3,$A3:$C9,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1456,19 +1387,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="2">
         <f>IF(A4&lt;&gt;"",IF(ROW()=3,$G2,E3),"")</f>
         <v/>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="2">
         <f>IF(A4&lt;&gt;"",TEXT(TIMEVALUE(D4)+(IFERROR(VLOOKUP(A4,$A3:$C9,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="2">
         <f>IF(A4&lt;&gt;"",IFERROR(VLOOKUP(A4,$A3:$C9,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1484,19 +1414,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="2">
         <f>IF(A5&lt;&gt;"",IF(ROW()=3,$G2,E4),"")</f>
         <v/>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="2">
         <f>IF(A5&lt;&gt;"",TEXT(TIMEVALUE(D5)+(IFERROR(VLOOKUP(A5,$A3:$C9,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="2">
         <f>IF(A5&lt;&gt;"",IFERROR(VLOOKUP(A5,$A3:$C9,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1512,19 +1441,18 @@
           <t>cine</t>
         </is>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="2">
         <f>IF(A6&lt;&gt;"",IF(ROW()=3,$G2,E5),"")</f>
         <v/>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="2">
         <f>IF(A6&lt;&gt;"",TEXT(TIMEVALUE(D6)+(IFERROR(VLOOKUP(A6,$A3:$C9,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="2">
         <f>IF(A6&lt;&gt;"",IFERROR(VLOOKUP(A6,$A3:$C9,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1540,19 +1468,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="2">
         <f>IF(A7&lt;&gt;"",IF(ROW()=3,$G2,E6),"")</f>
         <v/>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="2">
         <f>IF(A7&lt;&gt;"",TEXT(TIMEVALUE(D7)+(IFERROR(VLOOKUP(A7,$A3:$C9,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="2">
         <f>IF(A7&lt;&gt;"",IFERROR(VLOOKUP(A7,$A3:$C9,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1568,19 +1495,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="2">
         <f>IF(A8&lt;&gt;"",IF(ROW()=3,$G2,E7),"")</f>
         <v/>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="2">
         <f>IF(A8&lt;&gt;"",TEXT(TIMEVALUE(D8)+(IFERROR(VLOOKUP(A8,$A3:$C9,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="2">
         <f>IF(A8&lt;&gt;"",IFERROR(VLOOKUP(A8,$A3:$C9,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1596,19 +1522,18 @@
           <t>cine</t>
         </is>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="2">
         <f>IF(A9&lt;&gt;"",IF(ROW()=3,$G2,E8),"")</f>
         <v/>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="2">
         <f>IF(A9&lt;&gt;"",TEXT(TIMEVALUE(D9)+(IFERROR(VLOOKUP(A9,$A3:$C9,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="2">
         <f>IF(A9&lt;&gt;"",IFERROR(VLOOKUP(A9,$A3:$C9,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G9" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1630,7 +1555,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1664,16 +1589,16 @@
           <t>Tipo Calc</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
@@ -1693,19 +1618,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <f>IF(A3&lt;&gt;"",IF(ROW()=3,$G2,E2),"")</f>
         <v/>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <f>IF(A3&lt;&gt;"",TEXT(TIMEVALUE(D3)+(IFERROR(VLOOKUP(A3,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="2">
         <f>IF(A3&lt;&gt;"",IFERROR(VLOOKUP(A3,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1721,19 +1645,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <f>IF(A4&lt;&gt;"",IF(ROW()=3,$G2,E3),"")</f>
         <v/>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <f>IF(A4&lt;&gt;"",TEXT(TIMEVALUE(D4)+(IFERROR(VLOOKUP(A4,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="2">
         <f>IF(A4&lt;&gt;"",IFERROR(VLOOKUP(A4,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1749,19 +1672,18 @@
           <t>revista</t>
         </is>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="2">
         <f>IF(A5&lt;&gt;"",IF(ROW()=3,$G2,E4),"")</f>
         <v/>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="2">
         <f>IF(A5&lt;&gt;"",TEXT(TIMEVALUE(D5)+(IFERROR(VLOOKUP(A5,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="2">
         <f>IF(A5&lt;&gt;"",IFERROR(VLOOKUP(A5,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1777,19 +1699,18 @@
           <t>salud</t>
         </is>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="2">
         <f>IF(A6&lt;&gt;"",IF(ROW()=3,$G2,E5),"")</f>
         <v/>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="2">
         <f>IF(A6&lt;&gt;"",TEXT(TIMEVALUE(D6)+(IFERROR(VLOOKUP(A6,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="2">
         <f>IF(A6&lt;&gt;"",IFERROR(VLOOKUP(A6,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1805,19 +1726,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="2">
         <f>IF(A7&lt;&gt;"",IF(ROW()=3,$G2,E6),"")</f>
         <v/>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="2">
         <f>IF(A7&lt;&gt;"",TEXT(TIMEVALUE(D7)+(IFERROR(VLOOKUP(A7,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="2">
         <f>IF(A7&lt;&gt;"",IFERROR(VLOOKUP(A7,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1833,19 +1753,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="2">
         <f>IF(A8&lt;&gt;"",IF(ROW()=3,$G2,E7),"")</f>
         <v/>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="2">
         <f>IF(A8&lt;&gt;"",TEXT(TIMEVALUE(D8)+(IFERROR(VLOOKUP(A8,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="2">
         <f>IF(A8&lt;&gt;"",IFERROR(VLOOKUP(A8,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1861,19 +1780,18 @@
           <t>infantil</t>
         </is>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="2">
         <f>IF(A9&lt;&gt;"",IF(ROW()=3,$G2,E8),"")</f>
         <v/>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="2">
         <f>IF(A9&lt;&gt;"",TEXT(TIMEVALUE(D9)+(IFERROR(VLOOKUP(A9,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="2">
         <f>IF(A9&lt;&gt;"",IFERROR(VLOOKUP(A9,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1889,19 +1807,18 @@
           <t>animacion</t>
         </is>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <f>IF(A10&lt;&gt;"",IF(ROW()=3,$G2,E9),"")</f>
         <v/>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="2">
         <f>IF(A10&lt;&gt;"",TEXT(TIMEVALUE(D10)+(IFERROR(VLOOKUP(A10,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="2">
         <f>IF(A10&lt;&gt;"",IFERROR(VLOOKUP(A10,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1917,19 +1834,18 @@
           <t>animacion</t>
         </is>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <f>IF(A11&lt;&gt;"",IF(ROW()=3,$G2,E10),"")</f>
         <v/>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="2">
         <f>IF(A11&lt;&gt;"",TEXT(TIMEVALUE(D11)+(IFERROR(VLOOKUP(A11,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="2">
         <f>IF(A11&lt;&gt;"",IFERROR(VLOOKUP(A11,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1945,19 +1861,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="2">
         <f>IF(A12&lt;&gt;"",IF(ROW()=3,$G2,E11),"")</f>
         <v/>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="2">
         <f>IF(A12&lt;&gt;"",TEXT(TIMEVALUE(D12)+(IFERROR(VLOOKUP(A12,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F12" s="7">
+      <c r="F12" s="2">
         <f>IF(A12&lt;&gt;"",IFERROR(VLOOKUP(A12,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1973,19 +1888,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="2">
         <f>IF(A13&lt;&gt;"",IF(ROW()=3,$G2,E12),"")</f>
         <v/>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="2">
         <f>IF(A13&lt;&gt;"",TEXT(TIMEVALUE(D13)+(IFERROR(VLOOKUP(A13,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="2">
         <f>IF(A13&lt;&gt;"",IFERROR(VLOOKUP(A13,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2001,19 +1915,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="2">
         <f>IF(A14&lt;&gt;"",IF(ROW()=3,$G2,E13),"")</f>
         <v/>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="2">
         <f>IF(A14&lt;&gt;"",TEXT(TIMEVALUE(D14)+(IFERROR(VLOOKUP(A14,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="2">
         <f>IF(A14&lt;&gt;"",IFERROR(VLOOKUP(A14,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2029,19 +1942,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="2">
         <f>IF(A15&lt;&gt;"",IF(ROW()=3,$G2,E14),"")</f>
         <v/>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="2">
         <f>IF(A15&lt;&gt;"",TEXT(TIMEVALUE(D15)+(IFERROR(VLOOKUP(A15,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="2">
         <f>IF(A15&lt;&gt;"",IFERROR(VLOOKUP(A15,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2057,19 +1969,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="2">
         <f>IF(A16&lt;&gt;"",IF(ROW()=3,$G2,E15),"")</f>
         <v/>
       </c>
-      <c r="E16" s="3">
+      <c r="E16" s="2">
         <f>IF(A16&lt;&gt;"",TEXT(TIMEVALUE(D16)+(IFERROR(VLOOKUP(A16,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="2">
         <f>IF(A16&lt;&gt;"",IFERROR(VLOOKUP(A16,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2085,19 +1996,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="2">
         <f>IF(A17&lt;&gt;"",IF(ROW()=3,$G2,E16),"")</f>
         <v/>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="2">
         <f>IF(A17&lt;&gt;"",TEXT(TIMEVALUE(D17)+(IFERROR(VLOOKUP(A17,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F17" s="3">
+      <c r="F17" s="2">
         <f>IF(A17&lt;&gt;"",IFERROR(VLOOKUP(A17,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2113,19 +2023,18 @@
           <t>ficción</t>
         </is>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="2">
         <f>IF(A18&lt;&gt;"",IF(ROW()=3,$G2,E17),"")</f>
         <v/>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="2">
         <f>IF(A18&lt;&gt;"",TEXT(TIMEVALUE(D18)+(IFERROR(VLOOKUP(A18,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="2">
         <f>IF(A18&lt;&gt;"",IFERROR(VLOOKUP(A18,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2141,19 +2050,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="2">
         <f>IF(A19&lt;&gt;"",IF(ROW()=3,$G2,E18),"")</f>
         <v/>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="2">
         <f>IF(A19&lt;&gt;"",TEXT(TIMEVALUE(D19)+(IFERROR(VLOOKUP(A19,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="2">
         <f>IF(A19&lt;&gt;"",IFERROR(VLOOKUP(A19,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2169,19 +2077,18 @@
           <t>ficción</t>
         </is>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="2">
         <f>IF(A20&lt;&gt;"",IF(ROW()=3,$G2,E19),"")</f>
         <v/>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="2">
         <f>IF(A20&lt;&gt;"",TEXT(TIMEVALUE(D20)+(IFERROR(VLOOKUP(A20,$A3:$C20,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="2">
         <f>IF(A20&lt;&gt;"",IFERROR(VLOOKUP(A20,$A3:$C20,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G20" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2203,7 +2110,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2237,16 +2144,16 @@
           <t>Tipo Calc</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
         <is>
           <t>16:30</t>
         </is>
@@ -2266,19 +2173,18 @@
           <t>documental</t>
         </is>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="2">
         <f>IF(A3&lt;&gt;"",IF(ROW()=3,$G2,E2),"")</f>
         <v/>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="2">
         <f>IF(A3&lt;&gt;"",TEXT(TIMEVALUE(D3)+(IFERROR(VLOOKUP(A3,$A3:$C14,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="2">
         <f>IF(A3&lt;&gt;"",IFERROR(VLOOKUP(A3,$A3:$C14,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2294,19 +2200,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="2">
         <f>IF(A4&lt;&gt;"",IF(ROW()=3,$G2,E3),"")</f>
         <v/>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="2">
         <f>IF(A4&lt;&gt;"",TEXT(TIMEVALUE(D4)+(IFERROR(VLOOKUP(A4,$A3:$C14,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="2">
         <f>IF(A4&lt;&gt;"",IFERROR(VLOOKUP(A4,$A3:$C14,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2322,19 +2227,18 @@
           <t>cine</t>
         </is>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="2">
         <f>IF(A5&lt;&gt;"",IF(ROW()=3,$G2,E4),"")</f>
         <v/>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="2">
         <f>IF(A5&lt;&gt;"",TEXT(TIMEVALUE(D5)+(IFERROR(VLOOKUP(A5,$A3:$C14,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="2">
         <f>IF(A5&lt;&gt;"",IFERROR(VLOOKUP(A5,$A3:$C14,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2350,19 +2254,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="2">
         <f>IF(A6&lt;&gt;"",IF(ROW()=3,$G2,E5),"")</f>
         <v/>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="2">
         <f>IF(A6&lt;&gt;"",TEXT(TIMEVALUE(D6)+(IFERROR(VLOOKUP(A6,$A3:$C14,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="2">
         <f>IF(A6&lt;&gt;"",IFERROR(VLOOKUP(A6,$A3:$C14,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2378,19 +2281,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <f>IF(A7&lt;&gt;"",IF(ROW()=3,$G2,E6),"")</f>
         <v/>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="2">
         <f>IF(A7&lt;&gt;"",TEXT(TIMEVALUE(D7)+(IFERROR(VLOOKUP(A7,$A3:$C14,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="2">
         <f>IF(A7&lt;&gt;"",IFERROR(VLOOKUP(A7,$A3:$C14,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2406,19 +2308,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <f>IF(A8&lt;&gt;"",IF(ROW()=3,$G2,E7),"")</f>
         <v/>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="2">
         <f>IF(A8&lt;&gt;"",TEXT(TIMEVALUE(D8)+(IFERROR(VLOOKUP(A8,$A3:$C14,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="2">
         <f>IF(A8&lt;&gt;"",IFERROR(VLOOKUP(A8,$A3:$C14,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2434,19 +2335,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="2">
         <f>IF(A9&lt;&gt;"",IF(ROW()=3,$G2,E8),"")</f>
         <v/>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="2">
         <f>IF(A9&lt;&gt;"",TEXT(TIMEVALUE(D9)+(IFERROR(VLOOKUP(A9,$A3:$C14,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="2">
         <f>IF(A9&lt;&gt;"",IFERROR(VLOOKUP(A9,$A3:$C14,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2462,19 +2362,18 @@
           <t>entrevista</t>
         </is>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="2">
         <f>IF(A10&lt;&gt;"",IF(ROW()=3,$G2,E9),"")</f>
         <v/>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="2">
         <f>IF(A10&lt;&gt;"",TEXT(TIMEVALUE(D10)+(IFERROR(VLOOKUP(A10,$A3:$C14,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="2">
         <f>IF(A10&lt;&gt;"",IFERROR(VLOOKUP(A10,$A3:$C14,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2490,19 +2389,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="2">
         <f>IF(A11&lt;&gt;"",IF(ROW()=3,$G2,E10),"")</f>
         <v/>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="2">
         <f>IF(A11&lt;&gt;"",TEXT(TIMEVALUE(D11)+(IFERROR(VLOOKUP(A11,$A3:$C14,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="2">
         <f>IF(A11&lt;&gt;"",IFERROR(VLOOKUP(A11,$A3:$C14,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2518,19 +2416,18 @@
           <t>ficción</t>
         </is>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="2">
         <f>IF(A12&lt;&gt;"",IF(ROW()=3,$G2,E11),"")</f>
         <v/>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="2">
         <f>IF(A12&lt;&gt;"",TEXT(TIMEVALUE(D12)+(IFERROR(VLOOKUP(A12,$A3:$C14,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="2">
         <f>IF(A12&lt;&gt;"",IFERROR(VLOOKUP(A12,$A3:$C14,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2546,19 +2443,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="2">
         <f>IF(A13&lt;&gt;"",IF(ROW()=3,$G2,E12),"")</f>
         <v/>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="2">
         <f>IF(A13&lt;&gt;"",TEXT(TIMEVALUE(D13)+(IFERROR(VLOOKUP(A13,$A3:$C14,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="2">
         <f>IF(A13&lt;&gt;"",IFERROR(VLOOKUP(A13,$A3:$C14,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2574,19 +2470,18 @@
           <t>ficción</t>
         </is>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="2">
         <f>IF(A14&lt;&gt;"",IF(ROW()=3,$G2,E13),"")</f>
         <v/>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="2">
         <f>IF(A14&lt;&gt;"",TEXT(TIMEVALUE(D14)+(IFERROR(VLOOKUP(A14,$A3:$C14,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="2">
         <f>IF(A14&lt;&gt;"",IFERROR(VLOOKUP(A14,$A3:$C14,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G14" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2608,7 +2503,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2642,16 +2537,16 @@
           <t>Tipo Calc</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
@@ -2671,19 +2566,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <f>IF(A3&lt;&gt;"",IF(ROW()=3,$G2,E2),"")</f>
         <v/>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <f>IF(A3&lt;&gt;"",TEXT(TIMEVALUE(D3)+(IFERROR(VLOOKUP(A3,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="2">
         <f>IF(A3&lt;&gt;"",IFERROR(VLOOKUP(A3,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2699,19 +2593,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <f>IF(A4&lt;&gt;"",IF(ROW()=3,$G2,E3),"")</f>
         <v/>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <f>IF(A4&lt;&gt;"",TEXT(TIMEVALUE(D4)+(IFERROR(VLOOKUP(A4,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="2">
         <f>IF(A4&lt;&gt;"",IFERROR(VLOOKUP(A4,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2727,19 +2620,18 @@
           <t>infantil</t>
         </is>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="2">
         <f>IF(A5&lt;&gt;"",IF(ROW()=3,$G2,E4),"")</f>
         <v/>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="2">
         <f>IF(A5&lt;&gt;"",TEXT(TIMEVALUE(D5)+(IFERROR(VLOOKUP(A5,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="2">
         <f>IF(A5&lt;&gt;"",IFERROR(VLOOKUP(A5,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2755,19 +2647,18 @@
           <t>cine</t>
         </is>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="2">
         <f>IF(A6&lt;&gt;"",IF(ROW()=3,$G2,E5),"")</f>
         <v/>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="2">
         <f>IF(A6&lt;&gt;"",TEXT(TIMEVALUE(D6)+(IFERROR(VLOOKUP(A6,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="2">
         <f>IF(A6&lt;&gt;"",IFERROR(VLOOKUP(A6,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2783,19 +2674,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="2">
         <f>IF(A7&lt;&gt;"",IF(ROW()=3,$G2,E6),"")</f>
         <v/>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="2">
         <f>IF(A7&lt;&gt;"",TEXT(TIMEVALUE(D7)+(IFERROR(VLOOKUP(A7,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="2">
         <f>IF(A7&lt;&gt;"",IFERROR(VLOOKUP(A7,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2811,19 +2701,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="2">
         <f>IF(A8&lt;&gt;"",IF(ROW()=3,$G2,E7),"")</f>
         <v/>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="2">
         <f>IF(A8&lt;&gt;"",TEXT(TIMEVALUE(D8)+(IFERROR(VLOOKUP(A8,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="2">
         <f>IF(A8&lt;&gt;"",IFERROR(VLOOKUP(A8,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2839,19 +2728,18 @@
           <t>ficción</t>
         </is>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="2">
         <f>IF(A9&lt;&gt;"",IF(ROW()=3,$G2,E8),"")</f>
         <v/>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="2">
         <f>IF(A9&lt;&gt;"",TEXT(TIMEVALUE(D9)+(IFERROR(VLOOKUP(A9,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="2">
         <f>IF(A9&lt;&gt;"",IFERROR(VLOOKUP(A9,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2867,19 +2755,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="2">
         <f>IF(A10&lt;&gt;"",IF(ROW()=3,$G2,E9),"")</f>
         <v/>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="2">
         <f>IF(A10&lt;&gt;"",TEXT(TIMEVALUE(D10)+(IFERROR(VLOOKUP(A10,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="2">
         <f>IF(A10&lt;&gt;"",IFERROR(VLOOKUP(A10,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2895,19 +2782,18 @@
           <t>deporte</t>
         </is>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="2">
         <f>IF(A11&lt;&gt;"",IF(ROW()=3,$G2,E10),"")</f>
         <v/>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="2">
         <f>IF(A11&lt;&gt;"",TEXT(TIMEVALUE(D11)+(IFERROR(VLOOKUP(A11,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="2">
         <f>IF(A11&lt;&gt;"",IFERROR(VLOOKUP(A11,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2923,19 +2809,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="2">
         <f>IF(A12&lt;&gt;"",IF(ROW()=3,$G2,E11),"")</f>
         <v/>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="2">
         <f>IF(A12&lt;&gt;"",TEXT(TIMEVALUE(D12)+(IFERROR(VLOOKUP(A12,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="2">
         <f>IF(A12&lt;&gt;"",IFERROR(VLOOKUP(A12,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2951,19 +2836,18 @@
           <t>cine</t>
         </is>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="2">
         <f>IF(A13&lt;&gt;"",IF(ROW()=3,$G2,E12),"")</f>
         <v/>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="2">
         <f>IF(A13&lt;&gt;"",TEXT(TIMEVALUE(D13)+(IFERROR(VLOOKUP(A13,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="2">
         <f>IF(A13&lt;&gt;"",IFERROR(VLOOKUP(A13,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2979,19 +2863,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="2">
         <f>IF(A14&lt;&gt;"",IF(ROW()=3,$G2,E13),"")</f>
         <v/>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="2">
         <f>IF(A14&lt;&gt;"",TEXT(TIMEVALUE(D14)+(IFERROR(VLOOKUP(A14,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="2">
         <f>IF(A14&lt;&gt;"",IFERROR(VLOOKUP(A14,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3007,19 +2890,18 @@
           <t>animacion</t>
         </is>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="2">
         <f>IF(A15&lt;&gt;"",IF(ROW()=3,$G2,E14),"")</f>
         <v/>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="2">
         <f>IF(A15&lt;&gt;"",TEXT(TIMEVALUE(D15)+(IFERROR(VLOOKUP(A15,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="2">
         <f>IF(A15&lt;&gt;"",IFERROR(VLOOKUP(A15,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -3035,19 +2917,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="2">
         <f>IF(A16&lt;&gt;"",IF(ROW()=3,$G2,E15),"")</f>
         <v/>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="2">
         <f>IF(A16&lt;&gt;"",TEXT(TIMEVALUE(D16)+(IFERROR(VLOOKUP(A16,$A3:$C16,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="2">
         <f>IF(A16&lt;&gt;"",IFERROR(VLOOKUP(A16,$A3:$C16,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G16" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3069,7 +2950,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3103,16 +2984,16 @@
           <t>Tipo Calc</t>
         </is>
       </c>
-      <c r="G1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
         <is>
           <t>02:00</t>
         </is>
@@ -3132,19 +3013,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <f>IF(A3&lt;&gt;"",IF(ROW()=3,$G2,E2),"")</f>
         <v/>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="2">
         <f>IF(A3&lt;&gt;"",TEXT(TIMEVALUE(D3)+(IFERROR(VLOOKUP(A3,$A3:$C13,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="2">
         <f>IF(A3&lt;&gt;"",IFERROR(VLOOKUP(A3,$A3:$C13,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3160,19 +3040,18 @@
           <t>informativo</t>
         </is>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <f>IF(A4&lt;&gt;"",IF(ROW()=3,$G2,E3),"")</f>
         <v/>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="2">
         <f>IF(A4&lt;&gt;"",TEXT(TIMEVALUE(D4)+(IFERROR(VLOOKUP(A4,$A3:$C13,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="2">
         <f>IF(A4&lt;&gt;"",IFERROR(VLOOKUP(A4,$A3:$C13,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3188,19 +3067,18 @@
           <t>deporte</t>
         </is>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="2">
         <f>IF(A5&lt;&gt;"",IF(ROW()=3,$G2,E4),"")</f>
         <v/>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="2">
         <f>IF(A5&lt;&gt;"",TEXT(TIMEVALUE(D5)+(IFERROR(VLOOKUP(A5,$A3:$C13,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="2">
         <f>IF(A5&lt;&gt;"",IFERROR(VLOOKUP(A5,$A3:$C13,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3216,19 +3094,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="2">
         <f>IF(A6&lt;&gt;"",IF(ROW()=3,$G2,E5),"")</f>
         <v/>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="2">
         <f>IF(A6&lt;&gt;"",TEXT(TIMEVALUE(D6)+(IFERROR(VLOOKUP(A6,$A3:$C13,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="2">
         <f>IF(A6&lt;&gt;"",IFERROR(VLOOKUP(A6,$A3:$C13,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3244,19 +3121,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <f>IF(A7&lt;&gt;"",IF(ROW()=3,$G2,E6),"")</f>
         <v/>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="2">
         <f>IF(A7&lt;&gt;"",TEXT(TIMEVALUE(D7)+(IFERROR(VLOOKUP(A7,$A3:$C13,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="2">
         <f>IF(A7&lt;&gt;"",IFERROR(VLOOKUP(A7,$A3:$C13,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3272,19 +3148,18 @@
           <t>cultural</t>
         </is>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <f>IF(A8&lt;&gt;"",IF(ROW()=3,$G2,E7),"")</f>
         <v/>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="2">
         <f>IF(A8&lt;&gt;"",TEXT(TIMEVALUE(D8)+(IFERROR(VLOOKUP(A8,$A3:$C13,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="2">
         <f>IF(A8&lt;&gt;"",IFERROR(VLOOKUP(A8,$A3:$C13,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3300,19 +3175,18 @@
           <t>documental</t>
         </is>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <f>IF(A9&lt;&gt;"",IF(ROW()=3,$G2,E8),"")</f>
         <v/>
       </c>
-      <c r="E9" s="3">
+      <c r="E9" s="2">
         <f>IF(A9&lt;&gt;"",TEXT(TIMEVALUE(D9)+(IFERROR(VLOOKUP(A9,$A3:$C13,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="2">
         <f>IF(A9&lt;&gt;"",IFERROR(VLOOKUP(A9,$A3:$C13,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -3328,19 +3202,18 @@
           <t>documental</t>
         </is>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <f>IF(A10&lt;&gt;"",IF(ROW()=3,$G2,E9),"")</f>
         <v/>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="2">
         <f>IF(A10&lt;&gt;"",TEXT(TIMEVALUE(D10)+(IFERROR(VLOOKUP(A10,$A3:$C13,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="2">
         <f>IF(A10&lt;&gt;"",IFERROR(VLOOKUP(A10,$A3:$C13,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -3356,19 +3229,18 @@
           <t>entrevista</t>
         </is>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="2">
         <f>IF(A11&lt;&gt;"",IF(ROW()=3,$G2,E10),"")</f>
         <v/>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="2">
         <f>IF(A11&lt;&gt;"",TEXT(TIMEVALUE(D11)+(IFERROR(VLOOKUP(A11,$A3:$C13,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="2">
         <f>IF(A11&lt;&gt;"",IFERROR(VLOOKUP(A11,$A3:$C13,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -3384,19 +3256,18 @@
           <t>musical</t>
         </is>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="2">
         <f>IF(A12&lt;&gt;"",IF(ROW()=3,$G2,E11),"")</f>
         <v/>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="2">
         <f>IF(A12&lt;&gt;"",TEXT(TIMEVALUE(D12)+(IFERROR(VLOOKUP(A12,$A3:$C13,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="2">
         <f>IF(A12&lt;&gt;"",IFERROR(VLOOKUP(A12,$A3:$C13,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3412,19 +3283,18 @@
           <t>cine</t>
         </is>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="2">
         <f>IF(A13&lt;&gt;"",IF(ROW()=3,$G2,E12),"")</f>
         <v/>
       </c>
-      <c r="E13" s="4">
+      <c r="E13" s="2">
         <f>IF(A13&lt;&gt;"",TEXT(TIMEVALUE(D13)+(IFERROR(VLOOKUP(A13,$A3:$C13,2,FALSE),0)/1440),"hh:mm"),"")</f>
         <v/>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="2">
         <f>IF(A13&lt;&gt;"",IFERROR(VLOOKUP(A13,$A3:$C13,3,FALSE),0),"")</f>
         <v/>
       </c>
-      <c r="G13" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3437,7 +3307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3473,6 +3343,7 @@
           <t>Fin</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3492,6 +3363,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3511,6 +3383,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -3530,6 +3403,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -3549,6 +3423,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -3568,6 +3443,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -3587,6 +3463,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -3606,6 +3483,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3621,6 +3499,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>